<commit_message>
Sponsors: randomize order on each page load
</commit_message>
<xml_diff>
--- a/output/schedule_example.xlsx
+++ b/output/schedule_example.xlsx
@@ -822,12 +822,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>
@@ -1073,17 +1073,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>
@@ -1105,17 +1105,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1538,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Welkom: sponsor marquee strip beside Hoe reserveren (2/3 + 1/3 layout)
</commit_message>
<xml_diff>
--- a/output/schedule_example.xlsx
+++ b/output/schedule_example.xlsx
@@ -822,12 +822,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>
@@ -1073,17 +1073,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>
@@ -1105,17 +1105,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Eve B. &amp; Frank T.</t>
+          <t>Carol L. &amp; David P.</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1538,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Carol L. &amp; David P.</t>
+          <t>Eve B. &amp; Frank T.</t>
         </is>
       </c>
     </row>

</xml_diff>